<commit_message>
Fix all Sub Unit Kerja
</commit_message>
<xml_diff>
--- a/ref/Referensi-unor-dengan-parent-id.xlsx
+++ b/ref/Referensi-unor-dengan-parent-id.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dinaskominfo/kiken/Project/next/e-office2026/ref/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8EB7828-E7B7-DA42-9784-659E33D57447}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C4C590E-7349-6A47-9437-3BBDAE528E81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15740" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18267,7 +18267,7 @@
       <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="6" t="s">
         <v>2</v>
       </c>
       <c r="D1" t="s">
@@ -23181,10 +23181,10 @@
       </c>
     </row>
     <row r="247" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A247" t="s">
+      <c r="A247" s="6" t="s">
         <v>249</v>
       </c>
-      <c r="B247" t="s">
+      <c r="B247" s="6" t="s">
         <v>3545</v>
       </c>
       <c r="D247" s="5" t="s">
@@ -51839,7 +51839,7 @@
       <c r="C1" t="s">
         <v>1682</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="6" t="s">
         <v>1683</v>
       </c>
     </row>
@@ -56380,7 +56380,7 @@
       </c>
     </row>
     <row r="326" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A326" t="s">
+      <c r="A326" s="6" t="s">
         <v>2328</v>
       </c>
       <c r="B326">

</xml_diff>